<commit_message>
updated code version reporting
</commit_message>
<xml_diff>
--- a/downloads/Livraison 26-03-2026.1_updated-with-order.xlsx
+++ b/downloads/Livraison 26-03-2026.1_updated-with-order.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1547" uniqueCount="216">
   <si>
     <t>Tournée</t>
   </si>
@@ -82,7 +82,7 @@
     <t>MASY GERTINE</t>
   </si>
   <si>
-    <t>Gdp.deplog@galana.mg</t>
+    <t>alanic.nguetsa@camtrack.net</t>
   </si>
   <si>
     <t>Parking DEPOT TOLIARA</t>
@@ -1054,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S90"/>
+  <dimension ref="A1:S94"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13.07" customWidth="1"/>
@@ -6384,6 +6384,242 @@
         <v>19</v>
       </c>
     </row>
+    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>19</v>
+      </c>
+      <c r="B91" t="s">
+        <v>19</v>
+      </c>
+      <c r="C91" t="s">
+        <v>19</v>
+      </c>
+      <c r="D91" t="s">
+        <v>19</v>
+      </c>
+      <c r="E91" t="s">
+        <v>19</v>
+      </c>
+      <c r="F91" t="s">
+        <v>19</v>
+      </c>
+      <c r="G91" t="s">
+        <v>19</v>
+      </c>
+      <c r="H91" t="s">
+        <v>19</v>
+      </c>
+      <c r="I91" t="s">
+        <v>19</v>
+      </c>
+      <c r="J91" t="s">
+        <v>19</v>
+      </c>
+      <c r="K91" t="s">
+        <v>19</v>
+      </c>
+      <c r="L91" t="s">
+        <v>19</v>
+      </c>
+      <c r="M91" t="s">
+        <v>19</v>
+      </c>
+      <c r="N91" t="s">
+        <v>19</v>
+      </c>
+      <c r="O91" t="s">
+        <v>19</v>
+      </c>
+      <c r="P91" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>19</v>
+      </c>
+      <c r="R91" t="s">
+        <v>19</v>
+      </c>
+      <c r="S91" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>19</v>
+      </c>
+      <c r="B92" t="s">
+        <v>19</v>
+      </c>
+      <c r="C92" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" t="s">
+        <v>19</v>
+      </c>
+      <c r="E92" t="s">
+        <v>19</v>
+      </c>
+      <c r="F92" t="s">
+        <v>19</v>
+      </c>
+      <c r="G92" t="s">
+        <v>19</v>
+      </c>
+      <c r="H92" t="s">
+        <v>19</v>
+      </c>
+      <c r="I92" t="s">
+        <v>19</v>
+      </c>
+      <c r="J92" t="s">
+        <v>19</v>
+      </c>
+      <c r="K92" t="s">
+        <v>19</v>
+      </c>
+      <c r="L92" t="s">
+        <v>19</v>
+      </c>
+      <c r="M92" t="s">
+        <v>19</v>
+      </c>
+      <c r="N92" t="s">
+        <v>19</v>
+      </c>
+      <c r="O92" t="s">
+        <v>19</v>
+      </c>
+      <c r="P92" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>19</v>
+      </c>
+      <c r="R92" t="s">
+        <v>19</v>
+      </c>
+      <c r="S92" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>19</v>
+      </c>
+      <c r="B93" t="s">
+        <v>19</v>
+      </c>
+      <c r="C93" t="s">
+        <v>19</v>
+      </c>
+      <c r="D93" t="s">
+        <v>19</v>
+      </c>
+      <c r="E93" t="s">
+        <v>19</v>
+      </c>
+      <c r="F93" t="s">
+        <v>19</v>
+      </c>
+      <c r="G93" t="s">
+        <v>19</v>
+      </c>
+      <c r="H93" t="s">
+        <v>19</v>
+      </c>
+      <c r="I93" t="s">
+        <v>19</v>
+      </c>
+      <c r="J93" t="s">
+        <v>19</v>
+      </c>
+      <c r="K93" t="s">
+        <v>19</v>
+      </c>
+      <c r="L93" t="s">
+        <v>19</v>
+      </c>
+      <c r="M93" t="s">
+        <v>19</v>
+      </c>
+      <c r="N93" t="s">
+        <v>19</v>
+      </c>
+      <c r="O93" t="s">
+        <v>19</v>
+      </c>
+      <c r="P93" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>19</v>
+      </c>
+      <c r="R93" t="s">
+        <v>19</v>
+      </c>
+      <c r="S93" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>19</v>
+      </c>
+      <c r="B94" t="s">
+        <v>19</v>
+      </c>
+      <c r="C94" t="s">
+        <v>19</v>
+      </c>
+      <c r="D94" t="s">
+        <v>19</v>
+      </c>
+      <c r="E94" t="s">
+        <v>19</v>
+      </c>
+      <c r="F94" t="s">
+        <v>19</v>
+      </c>
+      <c r="G94" t="s">
+        <v>19</v>
+      </c>
+      <c r="H94" t="s">
+        <v>19</v>
+      </c>
+      <c r="I94" t="s">
+        <v>19</v>
+      </c>
+      <c r="J94" t="s">
+        <v>19</v>
+      </c>
+      <c r="K94" t="s">
+        <v>19</v>
+      </c>
+      <c r="L94" t="s">
+        <v>19</v>
+      </c>
+      <c r="M94" t="s">
+        <v>19</v>
+      </c>
+      <c r="N94" t="s">
+        <v>19</v>
+      </c>
+      <c r="O94" t="s">
+        <v>19</v>
+      </c>
+      <c r="P94" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>19</v>
+      </c>
+      <c r="R94" t="s">
+        <v>19</v>
+      </c>
+      <c r="S94" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>